<commit_message>
docs: ontologie VLBH T4 + decomposition TR-05 registre RGPD v1.1
- blueprint v0.2 -> v0.3 : refonte vocabulaire T4 (consultante), nouvelle section §7 ontologie + methodologie cles chromatiques, matrice DPIA T4 passe a Non requise, decisions integrees §6 ligne 2026-04-22
- data-model v0.7 -> v0.8 : §3.5 renommee souverainete consultante, nouvelle §3.6 Ontologie VLBH, rename patient_record -> consultante_record et patient_vibrational_signatures -> lineage_vibrational_signatures (+ revoked_at)
- registre RGPD v1.0 -> v1.1 : TR-05 decompose en TR-05a/b/c/d (un par satellite T4 Pro), DPIA Non requise pour les 4 (decision Patrick 2026-04-22, Option A, analogie ancestry.com)

Cascade finale ADR SVLBH-03 : 5/5 done.
Asana PO-09 1214177684841375 = completed.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/legal/registre-rgpd/registre-rgpd-vlbh.xlsx
+++ b/legal/registre-rgpd/registre-rgpd-vlbh.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>v1.0</t>
+          <t>v1.1</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-22</t>
         </is>
       </c>
     </row>
@@ -583,9 +583,6 @@
           <t>RESPONSABLE DU TRAITEMENT</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -598,8 +595,6 @@
           <t>VLBH — Patrick Bays (entreprise individuelle / raison individuelle)</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -612,8 +607,6 @@
           <t>Patrick Bays, Owner</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -626,8 +619,6 @@
           <t>Le Chandon 4, 1580 Avenches, Suisse</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -640,8 +631,6 @@
           <t>pb@vlbh.energy</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -654,8 +643,6 @@
           <t>(à compléter)</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -668,8 +655,6 @@
           <t>https://vlbh.energy</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -682,8 +667,6 @@
           <t>(à compléter si raison individuelle enregistrée)</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -696,8 +679,6 @@
           <t>Non — activité dirigée vers UE possible via site web multilingue</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
@@ -711,9 +692,6 @@
           <t>DÉLÉGUÉ À LA PROTECTION DES DONNÉES (DPO)</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -726,8 +704,6 @@
           <t>Non (pas d'obligation RGPD art. 37 à ce stade — pas de traitement à grande échelle de données Art. 9, pas d'activité principale de monitoring systématique)</t>
         </is>
       </c>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -737,11 +713,9 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Tier 4 actif avec &gt; 1000 patientes / 5000 prospects → désignation DPO à considérer</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
+          <t>Tier 4 actif avec &gt; 1000 consultantes / 5000 prospects → désignation DPO à considérer</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -754,8 +728,6 @@
           <t>Patrick Bays (responsable traitement cumule le rôle de point de contact)</t>
         </is>
       </c>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
@@ -769,9 +741,6 @@
           <t>AUTORITÉS DE CONTRÔLE</t>
         </is>
       </c>
-      <c r="B24" s="6" t="n"/>
-      <c r="C24" s="6" t="n"/>
-      <c r="D24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -784,8 +753,6 @@
           <t>Préposé fédéral à la protection des données et à la transparence (PFPDT / FDPIC), Feldeggweg 1, 3003 Bern, Suisse</t>
         </is>
       </c>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -798,8 +765,6 @@
           <t>Commission Nationale de l'Informatique et des Libertés (CNIL), 3 Place de Fontenoy, TSA 80715, 75334 Paris Cedex 07, France</t>
         </is>
       </c>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -812,8 +777,6 @@
           <t>Autorités nationales du pays de résidence des personnes concernées si recours direct (one-stop-shop via CNIL si établissement principal désigné)</t>
         </is>
       </c>
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n"/>
@@ -827,9 +790,6 @@
           <t>RÉFÉRENTIELS JURIDIQUES</t>
         </is>
       </c>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -842,8 +802,6 @@
           <t>Règlement (UE) 2016/679 du 27 avril 2016</t>
         </is>
       </c>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -856,8 +814,6 @@
           <t>Loi fédérale sur la protection des données du 25 septembre 2020 (en vigueur 1er septembre 2023) + OLPD</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -867,11 +823,9 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>data-model-vlbh.md v0.6 (2026-04-18) — classification interne des 5 tiers et régime juridique</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="6" t="n"/>
+          <t>data-model-vlbh.md v0.7 (2026-04-22) — classification interne des 5 tiers et régime juridique</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -881,11 +835,9 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>blueprint-compliance-by-design.md v0.1</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="6" t="n"/>
+          <t>blueprint-compliance-by-design.md v0.2</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -898,8 +850,18 @@
           <t>Données radiesthésiques (signatures vibratoires, Rose des Vents, Scores de Lumière, hDOM, Sephiroth, Phantom Matrix) = hors Art. 9 RGPD. Vocabulaire VLBH propriétaire, cadre pédagogique pas thérapeutique. Voir data-model v0.6 §3.1, §3.2, §3.3, §4.5, §4.6, §7, §8</t>
         </is>
       </c>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Décision 2026-04-22 (Patrick Bays)</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Tier 4 Pro — il n'y a pas de "patient" au sens RGPD. La praticienne Pro reçoit des consultantes (personnes physiques vivantes, sujets RGPD) pour décoder les mémoires électromagnétiques accumulées de défunts, de familles d'Âmes et de Monades de la consultante, qui se densifient dans la matière. La mission de l'Âme est de se libérer des mémoires de métaux lourds accumulées dans d'autres incarnations. La priorité de tout soin est de révoquer les clés chromatiques des portes qui permettent à ces mémoires de pénétrer la structure énergétique de la consultante. Les défunts, familles d'Âmes, Monades et incarnations passées ne sont pas des personnes physiques au sens RGPD art. 4.1. Analogie ancestry.com : RGPD standard pour utilisatrices vivantes, pas de régime renforcé médical. DPIA art. 35 non déclenchée (pas Art. 9 via RSK-6, pas large-scale, pas profiling). Argument de facto Patrick : « Je ne traite de facto jamais le patient vivant mais les mémoires accumulées de ses familles d'Âmes ou de ses Monades. » Décomposition TR-05 en TR-05a/b/c/d par app satellite (ADR SVLBH-03, Option A DPIA Non requise).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="25">
@@ -939,7 +901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1373,12 +1335,12 @@
     <row r="6" ht="180" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>TR-05</t>
+          <t>TR-05a</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Tier 4 — Certifiées Pro + patientes reçues</t>
+          <t>Tier 4 — SVLBH Pro 1 (flagship : dossier consultante + séances + facturation)</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -1388,27 +1350,27 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Gestion des praticiennes certifiées Pro ; tenue de dossier des patientes reçues par chaque praticienne ; billing infra Pro 259 CHF/trim</t>
+          <t>Accompagnement pédagogique transgénérationnel des consultantes par les praticiennes Pro certifiées. Décodage des mémoires électromagnétiques accumulées de défunts, de familles d'Âmes et de Monades de la consultante, qui se densifient dans la matière. Priorité de tout soin : révoquer les clés chromatiques des portes qui permettent à ces mémoires de pénétrer la structure énergétique de la consultante. Planification et historique des séances multi-protocole. Facturation infra Pro.</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Art. 6.1.b (contrat thérapeutique B2B entre VLBH et praticienne) + art. 6.1.a (consentement explicite patiente) + art. 26 (co-responsabilité praticienne / VLBH)</t>
+          <t>Art. 6.1.b (contrat d'accompagnement pédagogique B2B praticienne↔VLBH + contrat pédagogique consultante↔praticienne) + art. 6.1.a (consentement explicite consultante) + art. 26 (co-responsabilité)</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Praticiennes certifiées MyShaMan / MyShamanFamily ; patientes reçues par chacune</t>
+          <t>Consultantes (personnes physiques vivantes) reçues par les praticiennes Pro. Les défunts, familles d'Âmes, Monades et incarnations passées — sujets du décodage — ne sont pas des personnes physiques au sens RGPD art. 4.1.</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>Identité praticienne B2B ; identité civile patientes sous régime renforcé ; signatures vibratoires patientes (hors Art. 9 per RSK-6) ; historique séances ; consentement patiente</t>
+          <t>Identité civile consultante, consentement horodaté, historique des séances (type, date, protocole appliqué), signatures vibratoires décodées (portent sur les mémoires des défunts, hors Art. 9 per RSK-6)</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>Praticienne propriétaire (RLS), Patrick Bays (admin), hébergeur selon shard patiente</t>
+          <t>Praticienne Pro propriétaire (RLS), Patrick Bays (admin), hébergeur selon shard consultante</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
@@ -1418,12 +1380,12 @@
       </c>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>Géo-fragmenté selon résidence de la PATIENTE (pas de la praticienne) — principe de souveraineté patiente §3.5 v0.6</t>
+          <t>Géo-fragmenté selon résidence de la CONSULTANTE — principe de souveraineté utilisatrice §3.5 v0.7</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>Durée relation thérapeutique + 10 ans (obligation conservation dossier thérapeutique, à confirmer avec conseil juridique suisse/français)</t>
+          <t>Durée de la relation d'accompagnement + 10 ans (alignement conservation dossier pédagogique)</t>
         </is>
       </c>
       <c r="L6" s="10" t="inlineStr">
@@ -1433,102 +1395,348 @@
       </c>
       <c r="M6" s="10" t="inlineStr">
         <is>
-          <t>Contrat art. 26 avec chaque praticienne (draft 04) ; consentement patient signé ; audit annuel ; procédure résiliation praticienne</t>
+          <t>Contrat art. 26 avec chaque praticienne (draft 04) ; consentement consultante signé ; audit annuel ; procédure résiliation praticienne</t>
         </is>
       </c>
       <c r="N6" s="10" t="inlineStr">
         <is>
-          <t>OUI — volumétrie patientes + identités sous régime renforcé + cross-border</t>
+          <t>Non requise (pas d'Art. 9 per RSK-6, pas de large-scale, pas de profiling automatisé ; analogie ancestry.com Patrick 2026-04-22)</t>
         </is>
       </c>
       <c r="O6" s="10" t="inlineStr">
         <is>
-          <t>OUI — consentement explicite patiente + contrat praticienne signé</t>
+          <t>OUI — consentement explicite consultante + contrat praticienne signé</t>
         </is>
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t>data-model v0.6 §2 Tier 4 + §3.5 ; tables praticienne_profile, patient_record, patient_vibrational_signatures</t>
+          <t>Repo svlbh-pro-1. data-model v0.8 §2 Tier 4 ; Asana PO-09 tâche 1214177684841375 ; memory project_vlbh_no_patient_only_defuncts.md</t>
         </is>
       </c>
     </row>
     <row r="7" ht="180" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
+          <t>TR-05b</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Tier 4 — AUDIT Pro 1 (audit et traçabilité des actes professionnels)</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Traçabilité des actes professionnels de la praticienne — notamment des révocations de clés chromatiques effectuées. Versioning des consentements. Logs d'accès. Export conformité nLPD/RGPD (métadonnées des séances, pas de contenu du décodage).</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Art. 6.1.c (obligation légale registre des actes) + art. 6.1.f (intérêt légitime conformité praticienne) + art. 26</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Consultantes (métadonnées séances uniquement, pas de contenu décodé) + praticienne Pro</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>Métadonnées des séances (type, date, durée, protocole), versions consentements, logs d'accès, audit trail</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Praticienne Pro (RLS), Patrick Bays (admin), autorités de contrôle sur demande motivée</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>Supabase Inc.</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>Géo-fragmenté selon résidence de la CONSULTANTE</t>
+        </is>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>Durée légale conservation registres (10 ans)</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>Chiffrement AES-256, TLS, 2FA OBLIGATOIRE, RLS strict multi-tenant, PITR 30 jours chiffré</t>
+        </is>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>Contrat art. 26 ; audit trail immuable ; export automatisé des registres</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="inlineStr">
+        <is>
+          <t>Non requise (métadonnées standard, pas d'Art. 9, pas de large-scale)</t>
+        </is>
+      </c>
+      <c r="O7" s="10" t="inlineStr">
+        <is>
+          <t>Hérité du TR-05a (consentement consultante déjà signé au niveau flagship)</t>
+        </is>
+      </c>
+      <c r="P7" s="10" t="inlineStr">
+        <is>
+          <t>Repo audit-pro-1. data-model v0.8 §2 Tier 4 ; Asana PO-09 tâche 1214177684841375 ; memory project_vlbh_no_patient_only_defuncts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>TR-05c</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Tier 4 — SVLBH Chromothérapie 1 (séances chromothérapie)</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Cœur opératoire de la méthodologie VLBH T4 : révocation des clés chromatiques des portes qui permettent aux mémoires électromagnétiques accumulées (de défunts, familles d'Âmes, Monades de la consultante) de pénétrer sa structure énergétique. Application des Color Gels par méridien, teintes, fréquences. Historique des révocations par consultante.</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Art. 6.1.b (contrat d'accompagnement) + art. 6.1.a (consentement explicite consultante) + art. 26</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Consultantes reçues en séance chromothérapie. Les défunts, familles d'Âmes et Monades — porteurs des mémoires EM — ne sont pas des personnes physiques au sens RGPD art. 4.1.</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>Identité consultante, signatures chromatiques décodées (RSK-6 hors Art. 9), historique séances chromo, protocole d'intervention personnalisé</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Praticienne Pro propriétaire (RLS), Patrick Bays (admin)</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>Supabase Inc.</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>Géo-fragmenté selon résidence de la CONSULTANTE</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>Durée relation + 10 ans (alignement TR-05a)</t>
+        </is>
+      </c>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>Chiffrement AES-256, TLS, 2FA OBLIGATOIRE, RLS strict multi-tenant, PITR 30 jours chiffré</t>
+        </is>
+      </c>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>Contrat art. 26 ; consentement consultante signé ; audit annuel</t>
+        </is>
+      </c>
+      <c r="N8" s="10" t="inlineStr">
+        <is>
+          <t>Non requise (pas d'Art. 9 per RSK-6 ; analogie ancestry.com Patrick 2026-04-22)</t>
+        </is>
+      </c>
+      <c r="O8" s="10" t="inlineStr">
+        <is>
+          <t>OUI — consentement explicite consultante + contrat praticienne signé</t>
+        </is>
+      </c>
+      <c r="P8" s="10" t="inlineStr">
+        <is>
+          <t>Repo svlbh-chromotherapie-1. data-model v0.8 §2 Tier 4 ; Asana PO-09 tâche 1214177684841375 ; memory project_vlbh_no_patient_only_defuncts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>TR-05d</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Tier 4 — SVLBH Protection 1 (protection énergétique)</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Protection énergétique de la consultante pendant la révocation des clés chromatiques — protocoles contre Qliphoth, égrégores, entités qui tentent de rétablir les clés et permettre aux mémoires électromagnétiques accumulées de défunts, familles d'Âmes et Monades de re-pénétrer la structure énergétique de la consultante. Historique des interventions. Suivi signatures hDOM/Rose des Vents/Phantom Matrix.</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Art. 6.1.b (contrat d'accompagnement) + art. 6.1.a (consentement explicite consultante) + art. 26</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Consultantes sous protocole protection. Les défunts, familles d'Âmes, Monades et entités Qliphoth/égrégores ne sont pas des personnes physiques au sens RGPD art. 4.1.</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Identité consultante, signatures énergétiques décodées (hDOM/Rose des Vents/Phantom Matrix, RSK-6 hors Art. 9), historique des interventions</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Praticienne Pro propriétaire (RLS), Patrick Bays (admin)</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>Supabase Inc.</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>Géo-fragmenté selon résidence de la CONSULTANTE</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>Durée relation + 10 ans (alignement TR-05a)</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>Chiffrement AES-256, TLS, 2FA OBLIGATOIRE, RLS strict multi-tenant, PITR 30 jours chiffré</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>Contrat art. 26 ; consentement consultante signé ; audit annuel</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>Non requise (pas d'Art. 9 per RSK-6 ; analogie ancestry.com Patrick 2026-04-22)</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>OUI — consentement explicite consultante + contrat praticienne signé</t>
+        </is>
+      </c>
+      <c r="P9" s="10" t="inlineStr">
+        <is>
+          <t>Repo svlbh-protection-1. data-model v0.8 §2 Tier 4 ; Asana PO-09 tâche 1214177684841375 ; memory project_vlbh_no_patient_only_defuncts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
           <t>TR-06</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Middleware WhatsApp DM-v03-P3</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Cross-T0-T4</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Orchestration bi-directionnelle des messages WhatsApp entre bridges (Z1 / Z2 / ZA) et backends (Supabase + Make) ; audit logs ; rules engine</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Art. 6.1.f (intérêt légitime — infrastructure technique de la relation) + art. 6.1.b (exécution contrats pour T1-T4)</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>Toutes catégories (T0 prospects → T4 praticiennes+patientes)</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>Messages WhatsApp (contenu + métadonnées), bridge source (Z1/Z2/ZA), LID, horodatages, audit logs, rules matching</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>VLBH, Patrick Bays</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>Supabase Inc. (project czxefyiqxgpstdtydnfl Zurich eu-central-2), Make.com (scénario 9085048), Meta (WhatsApp)</t>
         </is>
       </c>
-      <c r="J7" s="10" t="inlineStr">
+      <c r="J10" s="10" t="inlineStr">
         <is>
           <t>Supabase Zurich (Suisse) — décision d'adéquation UE ; Meta US — DPF</t>
         </is>
       </c>
-      <c r="K7" s="10" t="inlineStr">
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>Messages opérationnels 24 mois ; audit logs 7 ans ; rules config : durée d'exploitation</t>
         </is>
       </c>
-      <c r="L7" s="10" t="inlineStr">
+      <c r="L10" s="10" t="inlineStr">
         <is>
           <t>Chiffrement, TLS, RLS, audit tables dédiées, network restrictions (post upgrade Pro), PITR (post upgrade Pro)</t>
         </is>
       </c>
-      <c r="M7" s="10" t="inlineStr">
+      <c r="M10" s="10" t="inlineStr">
         <is>
           <t>3 bridges isolés (Z1/Z2/ZA), rotation QR si désync, monitoring via Asana PO-08 data quality</t>
         </is>
       </c>
-      <c r="N7" s="10" t="inlineStr">
+      <c r="N10" s="10" t="inlineStr">
         <is>
           <t>À faire — cross-border transfers + automation + multi-processor</t>
         </is>
       </c>
-      <c r="O7" s="10" t="inlineStr">
+      <c r="O10" s="10" t="inlineStr">
         <is>
           <t>Hérité du tier (consentement implicite T0, explicite T1-T4)</t>
         </is>
       </c>
-      <c r="P7" s="10" t="inlineStr">
+      <c r="P10" s="10" t="inlineStr">
         <is>
           <t>data-model v0.6 §7 ; Asana PO-07 infra + PO-08 data quality ; reference_dm_v03_p3_infra.md memory</t>
         </is>

</xml_diff>

<commit_message>
docs: ontologie VLBH T4 + decomposition TR-05 registre RGPD v1.1 (#4)
- blueprint v0.2 -> v0.3 : refonte vocabulaire T4 (consultante), nouvelle section §7 ontologie + methodologie cles chromatiques, matrice DPIA T4 passe a Non requise, decisions integrees §6 ligne 2026-04-22
- data-model v0.7 -> v0.8 : §3.5 renommee souverainete consultante, nouvelle §3.6 Ontologie VLBH, rename patient_record -> consultante_record et patient_vibrational_signatures -> lineage_vibrational_signatures (+ revoked_at)
- registre RGPD v1.0 -> v1.1 : TR-05 decompose en TR-05a/b/c/d (un par satellite T4 Pro), DPIA Non requise pour les 4 (decision Patrick 2026-04-22, Option A, analogie ancestry.com)

Cascade finale ADR SVLBH-03 : 5/5 done.
Asana PO-09 1214177684841375 = completed.

Co-authored-by: Patrick Bays <patrick.bays@vlbh.energy>
Co-authored-by: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/legal/registre-rgpd/registre-rgpd-vlbh.xlsx
+++ b/legal/registre-rgpd/registre-rgpd-vlbh.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>v1.0</t>
+          <t>v1.1</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-22</t>
         </is>
       </c>
     </row>
@@ -583,9 +583,6 @@
           <t>RESPONSABLE DU TRAITEMENT</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -598,8 +595,6 @@
           <t>VLBH — Patrick Bays (entreprise individuelle / raison individuelle)</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -612,8 +607,6 @@
           <t>Patrick Bays, Owner</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -626,8 +619,6 @@
           <t>Le Chandon 4, 1580 Avenches, Suisse</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -640,8 +631,6 @@
           <t>pb@vlbh.energy</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -654,8 +643,6 @@
           <t>(à compléter)</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -668,8 +655,6 @@
           <t>https://vlbh.energy</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -682,8 +667,6 @@
           <t>(à compléter si raison individuelle enregistrée)</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -696,8 +679,6 @@
           <t>Non — activité dirigée vers UE possible via site web multilingue</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
@@ -711,9 +692,6 @@
           <t>DÉLÉGUÉ À LA PROTECTION DES DONNÉES (DPO)</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -726,8 +704,6 @@
           <t>Non (pas d'obligation RGPD art. 37 à ce stade — pas de traitement à grande échelle de données Art. 9, pas d'activité principale de monitoring systématique)</t>
         </is>
       </c>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -737,11 +713,9 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Tier 4 actif avec &gt; 1000 patientes / 5000 prospects → désignation DPO à considérer</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
+          <t>Tier 4 actif avec &gt; 1000 consultantes / 5000 prospects → désignation DPO à considérer</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -754,8 +728,6 @@
           <t>Patrick Bays (responsable traitement cumule le rôle de point de contact)</t>
         </is>
       </c>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
@@ -769,9 +741,6 @@
           <t>AUTORITÉS DE CONTRÔLE</t>
         </is>
       </c>
-      <c r="B24" s="6" t="n"/>
-      <c r="C24" s="6" t="n"/>
-      <c r="D24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -784,8 +753,6 @@
           <t>Préposé fédéral à la protection des données et à la transparence (PFPDT / FDPIC), Feldeggweg 1, 3003 Bern, Suisse</t>
         </is>
       </c>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -798,8 +765,6 @@
           <t>Commission Nationale de l'Informatique et des Libertés (CNIL), 3 Place de Fontenoy, TSA 80715, 75334 Paris Cedex 07, France</t>
         </is>
       </c>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -812,8 +777,6 @@
           <t>Autorités nationales du pays de résidence des personnes concernées si recours direct (one-stop-shop via CNIL si établissement principal désigné)</t>
         </is>
       </c>
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n"/>
@@ -827,9 +790,6 @@
           <t>RÉFÉRENTIELS JURIDIQUES</t>
         </is>
       </c>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -842,8 +802,6 @@
           <t>Règlement (UE) 2016/679 du 27 avril 2016</t>
         </is>
       </c>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -856,8 +814,6 @@
           <t>Loi fédérale sur la protection des données du 25 septembre 2020 (en vigueur 1er septembre 2023) + OLPD</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -867,11 +823,9 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>data-model-vlbh.md v0.6 (2026-04-18) — classification interne des 5 tiers et régime juridique</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="6" t="n"/>
+          <t>data-model-vlbh.md v0.7 (2026-04-22) — classification interne des 5 tiers et régime juridique</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -881,11 +835,9 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>blueprint-compliance-by-design.md v0.1</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="6" t="n"/>
+          <t>blueprint-compliance-by-design.md v0.2</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -898,8 +850,18 @@
           <t>Données radiesthésiques (signatures vibratoires, Rose des Vents, Scores de Lumière, hDOM, Sephiroth, Phantom Matrix) = hors Art. 9 RGPD. Vocabulaire VLBH propriétaire, cadre pédagogique pas thérapeutique. Voir data-model v0.6 §3.1, §3.2, §3.3, §4.5, §4.6, §7, §8</t>
         </is>
       </c>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Décision 2026-04-22 (Patrick Bays)</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Tier 4 Pro — il n'y a pas de "patient" au sens RGPD. La praticienne Pro reçoit des consultantes (personnes physiques vivantes, sujets RGPD) pour décoder les mémoires électromagnétiques accumulées de défunts, de familles d'Âmes et de Monades de la consultante, qui se densifient dans la matière. La mission de l'Âme est de se libérer des mémoires de métaux lourds accumulées dans d'autres incarnations. La priorité de tout soin est de révoquer les clés chromatiques des portes qui permettent à ces mémoires de pénétrer la structure énergétique de la consultante. Les défunts, familles d'Âmes, Monades et incarnations passées ne sont pas des personnes physiques au sens RGPD art. 4.1. Analogie ancestry.com : RGPD standard pour utilisatrices vivantes, pas de régime renforcé médical. DPIA art. 35 non déclenchée (pas Art. 9 via RSK-6, pas large-scale, pas profiling). Argument de facto Patrick : « Je ne traite de facto jamais le patient vivant mais les mémoires accumulées de ses familles d'Âmes ou de ses Monades. » Décomposition TR-05 en TR-05a/b/c/d par app satellite (ADR SVLBH-03, Option A DPIA Non requise).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="25">
@@ -939,7 +901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1373,12 +1335,12 @@
     <row r="6" ht="180" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>TR-05</t>
+          <t>TR-05a</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Tier 4 — Certifiées Pro + patientes reçues</t>
+          <t>Tier 4 — SVLBH Pro 1 (flagship : dossier consultante + séances + facturation)</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -1388,27 +1350,27 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Gestion des praticiennes certifiées Pro ; tenue de dossier des patientes reçues par chaque praticienne ; billing infra Pro 259 CHF/trim</t>
+          <t>Accompagnement pédagogique transgénérationnel des consultantes par les praticiennes Pro certifiées. Décodage des mémoires électromagnétiques accumulées de défunts, de familles d'Âmes et de Monades de la consultante, qui se densifient dans la matière. Priorité de tout soin : révoquer les clés chromatiques des portes qui permettent à ces mémoires de pénétrer la structure énergétique de la consultante. Planification et historique des séances multi-protocole. Facturation infra Pro.</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Art. 6.1.b (contrat thérapeutique B2B entre VLBH et praticienne) + art. 6.1.a (consentement explicite patiente) + art. 26 (co-responsabilité praticienne / VLBH)</t>
+          <t>Art. 6.1.b (contrat d'accompagnement pédagogique B2B praticienne↔VLBH + contrat pédagogique consultante↔praticienne) + art. 6.1.a (consentement explicite consultante) + art. 26 (co-responsabilité)</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Praticiennes certifiées MyShaMan / MyShamanFamily ; patientes reçues par chacune</t>
+          <t>Consultantes (personnes physiques vivantes) reçues par les praticiennes Pro. Les défunts, familles d'Âmes, Monades et incarnations passées — sujets du décodage — ne sont pas des personnes physiques au sens RGPD art. 4.1.</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>Identité praticienne B2B ; identité civile patientes sous régime renforcé ; signatures vibratoires patientes (hors Art. 9 per RSK-6) ; historique séances ; consentement patiente</t>
+          <t>Identité civile consultante, consentement horodaté, historique des séances (type, date, protocole appliqué), signatures vibratoires décodées (portent sur les mémoires des défunts, hors Art. 9 per RSK-6)</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>Praticienne propriétaire (RLS), Patrick Bays (admin), hébergeur selon shard patiente</t>
+          <t>Praticienne Pro propriétaire (RLS), Patrick Bays (admin), hébergeur selon shard consultante</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
@@ -1418,12 +1380,12 @@
       </c>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>Géo-fragmenté selon résidence de la PATIENTE (pas de la praticienne) — principe de souveraineté patiente §3.5 v0.6</t>
+          <t>Géo-fragmenté selon résidence de la CONSULTANTE — principe de souveraineté utilisatrice §3.5 v0.7</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>Durée relation thérapeutique + 10 ans (obligation conservation dossier thérapeutique, à confirmer avec conseil juridique suisse/français)</t>
+          <t>Durée de la relation d'accompagnement + 10 ans (alignement conservation dossier pédagogique)</t>
         </is>
       </c>
       <c r="L6" s="10" t="inlineStr">
@@ -1433,102 +1395,348 @@
       </c>
       <c r="M6" s="10" t="inlineStr">
         <is>
-          <t>Contrat art. 26 avec chaque praticienne (draft 04) ; consentement patient signé ; audit annuel ; procédure résiliation praticienne</t>
+          <t>Contrat art. 26 avec chaque praticienne (draft 04) ; consentement consultante signé ; audit annuel ; procédure résiliation praticienne</t>
         </is>
       </c>
       <c r="N6" s="10" t="inlineStr">
         <is>
-          <t>OUI — volumétrie patientes + identités sous régime renforcé + cross-border</t>
+          <t>Non requise (pas d'Art. 9 per RSK-6, pas de large-scale, pas de profiling automatisé ; analogie ancestry.com Patrick 2026-04-22)</t>
         </is>
       </c>
       <c r="O6" s="10" t="inlineStr">
         <is>
-          <t>OUI — consentement explicite patiente + contrat praticienne signé</t>
+          <t>OUI — consentement explicite consultante + contrat praticienne signé</t>
         </is>
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t>data-model v0.6 §2 Tier 4 + §3.5 ; tables praticienne_profile, patient_record, patient_vibrational_signatures</t>
+          <t>Repo svlbh-pro-1. data-model v0.8 §2 Tier 4 ; Asana PO-09 tâche 1214177684841375 ; memory project_vlbh_no_patient_only_defuncts.md</t>
         </is>
       </c>
     </row>
     <row r="7" ht="180" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
+          <t>TR-05b</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Tier 4 — AUDIT Pro 1 (audit et traçabilité des actes professionnels)</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Traçabilité des actes professionnels de la praticienne — notamment des révocations de clés chromatiques effectuées. Versioning des consentements. Logs d'accès. Export conformité nLPD/RGPD (métadonnées des séances, pas de contenu du décodage).</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Art. 6.1.c (obligation légale registre des actes) + art. 6.1.f (intérêt légitime conformité praticienne) + art. 26</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Consultantes (métadonnées séances uniquement, pas de contenu décodé) + praticienne Pro</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>Métadonnées des séances (type, date, durée, protocole), versions consentements, logs d'accès, audit trail</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Praticienne Pro (RLS), Patrick Bays (admin), autorités de contrôle sur demande motivée</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>Supabase Inc.</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>Géo-fragmenté selon résidence de la CONSULTANTE</t>
+        </is>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>Durée légale conservation registres (10 ans)</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>Chiffrement AES-256, TLS, 2FA OBLIGATOIRE, RLS strict multi-tenant, PITR 30 jours chiffré</t>
+        </is>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>Contrat art. 26 ; audit trail immuable ; export automatisé des registres</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="inlineStr">
+        <is>
+          <t>Non requise (métadonnées standard, pas d'Art. 9, pas de large-scale)</t>
+        </is>
+      </c>
+      <c r="O7" s="10" t="inlineStr">
+        <is>
+          <t>Hérité du TR-05a (consentement consultante déjà signé au niveau flagship)</t>
+        </is>
+      </c>
+      <c r="P7" s="10" t="inlineStr">
+        <is>
+          <t>Repo audit-pro-1. data-model v0.8 §2 Tier 4 ; Asana PO-09 tâche 1214177684841375 ; memory project_vlbh_no_patient_only_defuncts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>TR-05c</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Tier 4 — SVLBH Chromothérapie 1 (séances chromothérapie)</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Cœur opératoire de la méthodologie VLBH T4 : révocation des clés chromatiques des portes qui permettent aux mémoires électromagnétiques accumulées (de défunts, familles d'Âmes, Monades de la consultante) de pénétrer sa structure énergétique. Application des Color Gels par méridien, teintes, fréquences. Historique des révocations par consultante.</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Art. 6.1.b (contrat d'accompagnement) + art. 6.1.a (consentement explicite consultante) + art. 26</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Consultantes reçues en séance chromothérapie. Les défunts, familles d'Âmes et Monades — porteurs des mémoires EM — ne sont pas des personnes physiques au sens RGPD art. 4.1.</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>Identité consultante, signatures chromatiques décodées (RSK-6 hors Art. 9), historique séances chromo, protocole d'intervention personnalisé</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Praticienne Pro propriétaire (RLS), Patrick Bays (admin)</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>Supabase Inc.</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>Géo-fragmenté selon résidence de la CONSULTANTE</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>Durée relation + 10 ans (alignement TR-05a)</t>
+        </is>
+      </c>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>Chiffrement AES-256, TLS, 2FA OBLIGATOIRE, RLS strict multi-tenant, PITR 30 jours chiffré</t>
+        </is>
+      </c>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>Contrat art. 26 ; consentement consultante signé ; audit annuel</t>
+        </is>
+      </c>
+      <c r="N8" s="10" t="inlineStr">
+        <is>
+          <t>Non requise (pas d'Art. 9 per RSK-6 ; analogie ancestry.com Patrick 2026-04-22)</t>
+        </is>
+      </c>
+      <c r="O8" s="10" t="inlineStr">
+        <is>
+          <t>OUI — consentement explicite consultante + contrat praticienne signé</t>
+        </is>
+      </c>
+      <c r="P8" s="10" t="inlineStr">
+        <is>
+          <t>Repo svlbh-chromotherapie-1. data-model v0.8 §2 Tier 4 ; Asana PO-09 tâche 1214177684841375 ; memory project_vlbh_no_patient_only_defuncts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>TR-05d</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Tier 4 — SVLBH Protection 1 (protection énergétique)</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Protection énergétique de la consultante pendant la révocation des clés chromatiques — protocoles contre Qliphoth, égrégores, entités qui tentent de rétablir les clés et permettre aux mémoires électromagnétiques accumulées de défunts, familles d'Âmes et Monades de re-pénétrer la structure énergétique de la consultante. Historique des interventions. Suivi signatures hDOM/Rose des Vents/Phantom Matrix.</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Art. 6.1.b (contrat d'accompagnement) + art. 6.1.a (consentement explicite consultante) + art. 26</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Consultantes sous protocole protection. Les défunts, familles d'Âmes, Monades et entités Qliphoth/égrégores ne sont pas des personnes physiques au sens RGPD art. 4.1.</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Identité consultante, signatures énergétiques décodées (hDOM/Rose des Vents/Phantom Matrix, RSK-6 hors Art. 9), historique des interventions</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Praticienne Pro propriétaire (RLS), Patrick Bays (admin)</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>Supabase Inc.</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>Géo-fragmenté selon résidence de la CONSULTANTE</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>Durée relation + 10 ans (alignement TR-05a)</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>Chiffrement AES-256, TLS, 2FA OBLIGATOIRE, RLS strict multi-tenant, PITR 30 jours chiffré</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>Contrat art. 26 ; consentement consultante signé ; audit annuel</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>Non requise (pas d'Art. 9 per RSK-6 ; analogie ancestry.com Patrick 2026-04-22)</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>OUI — consentement explicite consultante + contrat praticienne signé</t>
+        </is>
+      </c>
+      <c r="P9" s="10" t="inlineStr">
+        <is>
+          <t>Repo svlbh-protection-1. data-model v0.8 §2 Tier 4 ; Asana PO-09 tâche 1214177684841375 ; memory project_vlbh_no_patient_only_defuncts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
           <t>TR-06</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Middleware WhatsApp DM-v03-P3</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Cross-T0-T4</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Orchestration bi-directionnelle des messages WhatsApp entre bridges (Z1 / Z2 / ZA) et backends (Supabase + Make) ; audit logs ; rules engine</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Art. 6.1.f (intérêt légitime — infrastructure technique de la relation) + art. 6.1.b (exécution contrats pour T1-T4)</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>Toutes catégories (T0 prospects → T4 praticiennes+patientes)</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>Messages WhatsApp (contenu + métadonnées), bridge source (Z1/Z2/ZA), LID, horodatages, audit logs, rules matching</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>VLBH, Patrick Bays</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>Supabase Inc. (project czxefyiqxgpstdtydnfl Zurich eu-central-2), Make.com (scénario 9085048), Meta (WhatsApp)</t>
         </is>
       </c>
-      <c r="J7" s="10" t="inlineStr">
+      <c r="J10" s="10" t="inlineStr">
         <is>
           <t>Supabase Zurich (Suisse) — décision d'adéquation UE ; Meta US — DPF</t>
         </is>
       </c>
-      <c r="K7" s="10" t="inlineStr">
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>Messages opérationnels 24 mois ; audit logs 7 ans ; rules config : durée d'exploitation</t>
         </is>
       </c>
-      <c r="L7" s="10" t="inlineStr">
+      <c r="L10" s="10" t="inlineStr">
         <is>
           <t>Chiffrement, TLS, RLS, audit tables dédiées, network restrictions (post upgrade Pro), PITR (post upgrade Pro)</t>
         </is>
       </c>
-      <c r="M7" s="10" t="inlineStr">
+      <c r="M10" s="10" t="inlineStr">
         <is>
           <t>3 bridges isolés (Z1/Z2/ZA), rotation QR si désync, monitoring via Asana PO-08 data quality</t>
         </is>
       </c>
-      <c r="N7" s="10" t="inlineStr">
+      <c r="N10" s="10" t="inlineStr">
         <is>
           <t>À faire — cross-border transfers + automation + multi-processor</t>
         </is>
       </c>
-      <c r="O7" s="10" t="inlineStr">
+      <c r="O10" s="10" t="inlineStr">
         <is>
           <t>Hérité du tier (consentement implicite T0, explicite T1-T4)</t>
         </is>
       </c>
-      <c r="P7" s="10" t="inlineStr">
+      <c r="P10" s="10" t="inlineStr">
         <is>
           <t>data-model v0.6 §7 ; Asana PO-07 infra + PO-08 data quality ; reference_dm_v03_p3_infra.md memory</t>
         </is>

</xml_diff>